<commit_message>
docs: finalize UAV developer documentation package
</commit_message>
<xml_diff>
--- a/docs/非凸α-接口总表.xlsx
+++ b/docs/非凸α-接口总表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口总表" sheetId="1" r:id="Rc8063e171f93470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口总表" sheetId="1" r:id="Rc1aa8081fad1487a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -240,7 +240,6 @@
       <x:c r="P1" t="str">
         <x:v>source_path</x:v>
       </x:c>
-      <x:c r="Q1" t="str"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
@@ -291,7 +290,6 @@
       <x:c r="P2" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/run_single_lio.sh</x:v>
       </x:c>
-      <x:c r="Q2" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -342,7 +340,6 @@
       <x:c r="P3" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/run_single_vio.sh</x:v>
       </x:c>
-      <x:c r="Q3" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -393,7 +390,6 @@
       <x:c r="P4" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/takeoff.sh</x:v>
       </x:c>
-      <x:c r="Q4" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -444,7 +440,6 @@
       <x:c r="P5" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/pub_trigger.sh</x:v>
       </x:c>
-      <x:c r="Q5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
@@ -495,7 +490,6 @@
       <x:c r="P6" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/back.sh</x:v>
       </x:c>
-      <x:c r="Q6" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -546,7 +540,6 @@
       <x:c r="P7" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/land.sh</x:v>
       </x:c>
-      <x:c r="Q7" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
@@ -568,36 +561,33 @@
         <x:v>quadrotor_msgs/TakeoffLand</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>takeoff_land_cmd={1 takeoff</x:v>
+        <x:v>takeoff_land_cmd={1 takeoff,2 land}</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>2 land}</x:v>
+        <x:v>script or RC bridge</x:v>
       </x:c>
       <x:c r="I8" t="str">
-        <x:v>script or RC bridge</x:v>
+        <x:v>px4ctrl</x:v>
       </x:c>
       <x:c r="J8" t="str">
-        <x:v>px4ctrl</x:v>
+        <x:v>px4ctrl 与定位链正常</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>px4ctrl 与定位链正常</x:v>
+        <x:v>起飞与降落动作原语</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>起飞与降落动作原语</x:v>
+        <x:v>rostopic pub -1 /px4ctrl/takeoff_land quadrotor_msgs/TakeoffLand 'takeoff_land_cmd: 1'</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>rostopic pub -1 /px4ctrl/takeoff_land quadrotor_msgs/TakeoffLand 'takeoff_land_cmd: 1'</x:v>
+        <x:v>onboard-active</x:v>
       </x:c>
       <x:c r="N8" t="str">
-        <x:v>onboard-active</x:v>
+        <x:v>RC 档位不对会被拒绝</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>RC 档位不对会被拒绝</x:v>
+        <x:v>E008_takeoff_topic</x:v>
       </x:c>
       <x:c r="P8" t="str">
-        <x:v>E008_takeoff_topic</x:v>
-      </x:c>
-      <x:c r="Q8" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/sh_files/takeoff.sh</x:v>
       </x:c>
     </x:row>
@@ -650,7 +640,6 @@
       <x:c r="P9" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/src/multipointplan.cpp</x:v>
       </x:c>
-      <x:c r="Q9" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
@@ -701,7 +690,6 @@
       <x:c r="P10" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/src/multipointplan.cpp</x:v>
       </x:c>
-      <x:c r="Q10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
@@ -752,7 +740,6 @@
       <x:c r="P11" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/src/multipointplan.cpp</x:v>
       </x:c>
-      <x:c r="Q11" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
@@ -803,7 +790,6 @@
       <x:c r="P12" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/src/multipointplan.cpp</x:v>
       </x:c>
-      <x:c r="Q12" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -854,7 +840,6 @@
       <x:c r="P13" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/realflight_modules/px4ctrl/launch/run_ctrl_lio.launch</x:v>
       </x:c>
-      <x:c r="Q13" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
@@ -905,7 +890,6 @@
       <x:c r="P14" t="str">
         <x:v>uav/10-knowledge-base/06-指令速查-含隐藏命令.md</x:v>
       </x:c>
-      <x:c r="Q14" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
@@ -956,7 +940,6 @@
       <x:c r="P15" t="str">
         <x:v>uav/10-knowledge-base/05-传感器与状态回传.md</x:v>
       </x:c>
-      <x:c r="Q15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
@@ -1007,7 +990,6 @@
       <x:c r="P16" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/src/multipointplan.cpp</x:v>
       </x:c>
-      <x:c r="Q16" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
@@ -1058,7 +1040,6 @@
       <x:c r="P17" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/realflight_modules/px4ctrl/src/px4ctrl_node.cpp</x:v>
       </x:c>
-      <x:c r="Q17" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
@@ -1109,7 +1090,6 @@
       <x:c r="P18" t="str">
         <x:v>uav/10-knowledge-base/05-传感器与状态回传.md</x:v>
       </x:c>
-      <x:c r="Q18" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
@@ -1160,7 +1140,6 @@
       <x:c r="P19" t="str">
         <x:v>uav/10-knowledge-base/05-传感器与状态回传.md</x:v>
       </x:c>
-      <x:c r="Q19" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
@@ -1211,7 +1190,6 @@
       <x:c r="P20" t="str">
         <x:v>uav/10-knowledge-base/05-传感器与状态回传.md</x:v>
       </x:c>
-      <x:c r="Q20" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
@@ -1262,7 +1240,6 @@
       <x:c r="P21" t="str">
         <x:v>uav/10-knowledge-base/05-传感器与状态回传.md</x:v>
       </x:c>
-      <x:c r="Q21" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
@@ -1313,7 +1290,6 @@
       <x:c r="P22" t="str">
         <x:v>uav/10-knowledge-base/05-传感器与状态回传.md</x:v>
       </x:c>
-      <x:c r="Q22" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
@@ -1364,7 +1340,6 @@
       <x:c r="P23" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/diff_planner/plan_manage/launch/exp/run_exp_single_lio.launch</x:v>
       </x:c>
-      <x:c r="Q23" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
@@ -1415,7 +1390,6 @@
       <x:c r="P24" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/config/points.yaml</x:v>
       </x:c>
-      <x:c r="Q24" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
@@ -1466,7 +1440,6 @@
       <x:c r="P25" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/realflight_modules/px4ctrl/config/ctrl_param_fpv.yaml</x:v>
       </x:c>
-      <x:c r="Q25" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
@@ -1517,7 +1490,6 @@
       <x:c r="P26" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/launch/multipointplan_exp_lio.launch</x:v>
       </x:c>
-      <x:c r="Q26" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
@@ -1568,7 +1540,6 @@
       <x:c r="P27" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/diff_planner/plan_manage/launch/exp/run_exp_single_lio.launch</x:v>
       </x:c>
-      <x:c r="Q27" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
@@ -1619,7 +1590,6 @@
       <x:c r="P28" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/diff_planner/plan_manage/launch/exp/run_exp_single_vio.launch</x:v>
       </x:c>
-      <x:c r="Q28" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
@@ -1670,7 +1640,6 @@
       <x:c r="P29" t="str">
         <x:v>uav/10-knowledge-base/01-硬件与系统.md</x:v>
       </x:c>
-      <x:c r="Q29" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
@@ -1721,7 +1690,6 @@
       <x:c r="P30" t="str">
         <x:v>uav/10-knowledge-base/01-硬件与系统.md</x:v>
       </x:c>
-      <x:c r="Q30" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
@@ -1772,7 +1740,6 @@
       <x:c r="P31" t="str">
         <x:v>uav/10-knowledge-base/01-硬件与系统.md</x:v>
       </x:c>
-      <x:c r="Q31" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
@@ -1823,7 +1790,6 @@
       <x:c r="P32" t="str">
         <x:v>uav/03-drone-code/snapshot_20260421_174511/Diff-planner/src/user_command/multipoint/src/multipointplan.cpp</x:v>
       </x:c>
-      <x:c r="Q32" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>